<commit_message>
added render port config
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,21 +478,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Open Elective</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14:34:45.488369</t>
+          <t>09:10:58.248923</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -503,31 +503,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>059</t>
+          <t>055</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SOORAJ S</t>
+          <t>JANE MARIA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Software Testing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20:40:05.166791</t>
+          <t>11:51:47.375974</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -538,33 +538,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>040</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sanjay cu</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Indian Constitution</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12:01:34.425003</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>059</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>SOORAJ S</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>20:41:24.382962</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Indian Constitution</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12:02:30.240477</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>present</t>
         </is>

</xml_diff>